<commit_message>
correction of 2 algorithms
dis_msk_ever
dis_cvd_hbp_diag_or_med_ever
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-NES.xlsx
+++ b/baseline/data_processing_elements-NES.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/849507f40a0f895e/Documents/ProPASS/NES/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sbtiali\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{DBD72419-52E8-4439-AB9B-D71018BC44AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B1F98D7-3C1C-43A3-96D3-D44C78D7ED80}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5098D060-15A2-4ADF-9F0C-4987B471B465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0073E314-1B2C-4924-AC81-D526EEC9786A}"/>
   </bookViews>
@@ -2920,21 +2920,8 @@
     <t>The study-specific variable for self-reported myocardial infarction was used to assign positive responses for the DataSchema variables. Negative responses could not be assigned.</t>
   </si>
   <si>
-    <t>case_when(
-fq289 == 1 | fq319 == 1 | fq364 == 1 ~ 1L;
-fq289 == 0 &amp; fq319 == 0 &amp; fq364 ==0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
     <t>I think the study variables cover all the options, so can assign 0 if all 0.
 Can remove as.numeric.</t>
-  </si>
-  <si>
-    <t>case_when(
-fq241 == 1 | fq244 == 1 ~ 1L;
-fq241 == 0 &amp; fq244 == 0 ~ 0L;
-fq241 == 0 | fq244 == 0 ~ 2L;
-ELSE ~ NA_integer_)</t>
   </si>
   <si>
     <t>case_when(
@@ -3326,6 +3313,19 @@
     <t>case_when(year(questionnaire_date) == 2021 &amp; !is.na(body_fat_mass_kg) &amp; body_fat_mass_kg &gt; 0 ~ "Single-frequency analysis (1500, Bodystat, Douglas, Isle of Man)";
 year(questionnaire_date) &gt; 2021 &amp; !is.na(body_fat_mass_kg) &amp; body_fat_mass_kg &gt; 0~ "multi-frequency analysis (770, InBody, Seoul, South Korea)";
 ELSE ~ NA)</t>
+  </si>
+  <si>
+    <t>case_when(
+fq241 == 1 | fq244 == 1 ~ 1L;
+fq241 == 2 &amp; fq244 == 2 ~ 0L;
+fq241 == 2 | fq244 == 2 ~ 2L;
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>case_when(
+fq289 == 1 | fq319 == 1 | fq364 == 1 ~ 1L;
+fq289 == 2 &amp; fq319 == 2 &amp; fq364 ==0 ~ 0L ; 
+ELSE ~ NA_integer_)</t>
   </si>
 </sst>
 </file>
@@ -3481,10 +3481,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3904,10 +3900,10 @@
         <v>17</v>
       </c>
       <c r="U1" s="13" t="s">
-        <v>844</v>
+        <v>842</v>
       </c>
       <c r="V1" s="10" t="s">
-        <v>845</v>
+        <v>843</v>
       </c>
       <c r="W1" s="10" t="s">
         <v>18</v>
@@ -4144,7 +4140,7 @@
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>484</v>
@@ -4233,7 +4229,7 @@
         <v>493</v>
       </c>
       <c r="Y7" s="2" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
     </row>
     <row r="8" spans="1:32" ht="60" x14ac:dyDescent="0.25">
@@ -4404,13 +4400,13 @@
         <v>493</v>
       </c>
       <c r="Y10" s="2" t="s">
-        <v>881</v>
+        <v>879</v>
       </c>
       <c r="Z10" s="1" t="s">
         <v>507</v>
       </c>
       <c r="AB10" s="12" t="s">
-        <v>850</v>
+        <v>848</v>
       </c>
     </row>
     <row r="11" spans="1:32" ht="75" x14ac:dyDescent="0.25">
@@ -4475,10 +4471,10 @@
         <v>783</v>
       </c>
       <c r="AA11" s="15" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="AB11" s="12" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
     </row>
     <row r="12" spans="1:32" ht="75" x14ac:dyDescent="0.25">
@@ -4543,7 +4539,7 @@
         <v>785</v>
       </c>
       <c r="AA12" s="15" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="AB12" s="12" t="s">
         <v>790</v>
@@ -4596,7 +4592,7 @@
         <v>512</v>
       </c>
       <c r="U13" s="12" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="V13" s="11" t="s">
         <v>514</v>
@@ -4673,7 +4669,7 @@
         <v>786</v>
       </c>
       <c r="AA14" s="15" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="AB14" s="12" t="s">
         <v>790</v>
@@ -4726,7 +4722,7 @@
         <v>512</v>
       </c>
       <c r="U15" s="12" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="V15" s="11" t="s">
         <v>514</v>
@@ -4788,7 +4784,7 @@
         <v>512</v>
       </c>
       <c r="U16" s="12" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="V16" s="11" t="s">
         <v>514</v>
@@ -4850,7 +4846,7 @@
         <v>512</v>
       </c>
       <c r="U17" s="12" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="V17" s="11" t="s">
         <v>514</v>
@@ -4912,7 +4908,7 @@
         <v>512</v>
       </c>
       <c r="U18" s="12" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="V18" s="11" t="s">
         <v>514</v>
@@ -4974,7 +4970,7 @@
         <v>512</v>
       </c>
       <c r="U19" s="12" t="s">
-        <v>849</v>
+        <v>847</v>
       </c>
       <c r="V19" s="11" t="s">
         <v>474</v>
@@ -4989,7 +4985,7 @@
         <v>515</v>
       </c>
       <c r="AA19" s="15" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="AB19" s="12" t="s">
         <v>791</v>
@@ -5113,7 +5109,7 @@
         <v>560</v>
       </c>
       <c r="AB21" s="12" t="s">
-        <v>851</v>
+        <v>849</v>
       </c>
     </row>
     <row r="22" spans="1:28" ht="30" x14ac:dyDescent="0.25">
@@ -5172,7 +5168,7 @@
         <v>776</v>
       </c>
       <c r="AB22" s="12" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
     </row>
     <row r="23" spans="1:28" ht="180" x14ac:dyDescent="0.25">
@@ -5284,7 +5280,7 @@
         <v>527</v>
       </c>
       <c r="Y24" s="2" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="Z24" s="2" t="s">
         <v>540</v>
@@ -5838,7 +5834,7 @@
         <v>359</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
       <c r="V34" s="1" t="s">
         <v>474</v>
@@ -5850,7 +5846,7 @@
         <v>486</v>
       </c>
       <c r="Y34" s="1" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
     </row>
     <row r="35" spans="1:28" ht="195" x14ac:dyDescent="0.25">
@@ -5873,7 +5869,7 @@
         <v>349</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
       <c r="V35" s="1" t="s">
         <v>474</v>
@@ -5885,10 +5881,10 @@
         <v>527</v>
       </c>
       <c r="Y35" s="2" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="Z35" s="2" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
     </row>
     <row r="36" spans="1:28" ht="120" x14ac:dyDescent="0.25">
@@ -5938,7 +5934,7 @@
         <v>360</v>
       </c>
       <c r="U36" s="12" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="V36" s="1" t="s">
         <v>474</v>
@@ -5950,13 +5946,13 @@
         <v>486</v>
       </c>
       <c r="Y36" s="2" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
       <c r="Z36" s="2" t="s">
         <v>570</v>
       </c>
       <c r="AB36" s="12" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
     </row>
     <row r="37" spans="1:28" ht="120" x14ac:dyDescent="0.25">
@@ -6006,7 +6002,7 @@
         <v>360</v>
       </c>
       <c r="U37" s="12" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="V37" s="1" t="s">
         <v>474</v>
@@ -6018,13 +6014,13 @@
         <v>486</v>
       </c>
       <c r="Y37" s="2" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
       <c r="Z37" s="2" t="s">
         <v>570</v>
       </c>
       <c r="AB37" s="12" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
     </row>
     <row r="38" spans="1:28" ht="120" x14ac:dyDescent="0.25">
@@ -6074,7 +6070,7 @@
         <v>578</v>
       </c>
       <c r="U38" s="12" t="s">
-        <v>852</v>
+        <v>850</v>
       </c>
       <c r="V38" s="1" t="s">
         <v>474</v>
@@ -6086,13 +6082,13 @@
         <v>486</v>
       </c>
       <c r="Y38" s="12" t="s">
-        <v>854</v>
+        <v>852</v>
       </c>
       <c r="Z38" s="2" t="s">
         <v>570</v>
       </c>
       <c r="AB38" s="12" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
     </row>
     <row r="39" spans="1:28" ht="75" x14ac:dyDescent="0.25">
@@ -6136,7 +6132,7 @@
         <v>514</v>
       </c>
       <c r="AB39" s="12" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
     </row>
     <row r="40" spans="1:28" ht="105" x14ac:dyDescent="0.25">
@@ -6180,7 +6176,7 @@
         <v>584</v>
       </c>
       <c r="U40" s="12" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
       <c r="V40" s="1" t="s">
         <v>474</v>
@@ -6192,14 +6188,14 @@
         <v>493</v>
       </c>
       <c r="Y40" s="12" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
       <c r="Z40" s="2"/>
       <c r="AA40" s="15" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="AB40" s="12" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
     </row>
     <row r="41" spans="1:28" x14ac:dyDescent="0.25">
@@ -6334,7 +6330,7 @@
         <v>776</v>
       </c>
       <c r="AB43" s="12" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
     </row>
     <row r="44" spans="1:28" ht="30" x14ac:dyDescent="0.25">
@@ -6393,7 +6389,7 @@
         <v>776</v>
       </c>
       <c r="AB44" s="12" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
     </row>
     <row r="45" spans="1:28" ht="30" x14ac:dyDescent="0.25">
@@ -6452,7 +6448,7 @@
         <v>776</v>
       </c>
       <c r="AB45" s="12" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
     </row>
     <row r="46" spans="1:28" ht="120" x14ac:dyDescent="0.25">
@@ -6517,7 +6513,7 @@
         <v>602</v>
       </c>
       <c r="AB46" s="12" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
     </row>
     <row r="47" spans="1:28" ht="45" x14ac:dyDescent="0.25">
@@ -6576,7 +6572,7 @@
         <v>776</v>
       </c>
       <c r="AB47" s="12" t="s">
-        <v>858</v>
+        <v>856</v>
       </c>
     </row>
     <row r="48" spans="1:28" ht="30" x14ac:dyDescent="0.25">
@@ -6903,7 +6899,7 @@
         <v>760</v>
       </c>
       <c r="AB54" s="12" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
     </row>
     <row r="55" spans="1:28" ht="60" x14ac:dyDescent="0.25">
@@ -7072,7 +7068,7 @@
       </c>
       <c r="AA57" s="14"/>
       <c r="AB57" s="12" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
     </row>
     <row r="58" spans="1:28" ht="90" x14ac:dyDescent="0.25">
@@ -7134,7 +7130,7 @@
         <v>486</v>
       </c>
       <c r="Y58" s="2" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="Z58" s="2" t="s">
         <v>772</v>
@@ -7349,13 +7345,13 @@
         <v>638</v>
       </c>
       <c r="Y62" s="15" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="Z62" s="2" t="s">
         <v>773</v>
       </c>
       <c r="AB62" s="12" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
     </row>
     <row r="63" spans="1:28" ht="105" x14ac:dyDescent="0.25">
@@ -7535,7 +7531,7 @@
         <v>761</v>
       </c>
       <c r="AB65" s="12" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
     </row>
     <row r="66" spans="1:29" ht="45" x14ac:dyDescent="0.25">
@@ -7635,13 +7631,13 @@
         <v>638</v>
       </c>
       <c r="Y67" s="15" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="Z67" s="2" t="s">
         <v>650</v>
       </c>
       <c r="AB67" s="12" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
     </row>
     <row r="68" spans="1:29" ht="255" x14ac:dyDescent="0.25">
@@ -7704,7 +7700,7 @@
       </c>
       <c r="AA68" s="1"/>
       <c r="AB68" s="12" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
     </row>
     <row r="69" spans="1:29" ht="255" x14ac:dyDescent="0.25">
@@ -7763,7 +7759,7 @@
         <v>514</v>
       </c>
       <c r="AB69" s="12" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
     </row>
     <row r="70" spans="1:29" ht="60" x14ac:dyDescent="0.25">
@@ -7869,7 +7865,7 @@
         <v>663</v>
       </c>
       <c r="U71" s="12" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="V71" s="1" t="s">
         <v>474</v>
@@ -7887,7 +7883,7 @@
         <v>666</v>
       </c>
       <c r="AB71" s="1" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
     </row>
     <row r="72" spans="1:29" ht="90" x14ac:dyDescent="0.25">
@@ -7916,7 +7912,7 @@
         <v>446</v>
       </c>
       <c r="L72" s="1" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="M72" s="2" t="s">
         <v>667</v>
@@ -7947,19 +7943,19 @@
         <v>493</v>
       </c>
       <c r="Y72" s="2" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="Z72" s="2" t="s">
         <v>774</v>
       </c>
       <c r="AA72" s="2" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
       <c r="AB72" s="2" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
       <c r="AC72" s="1" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
     </row>
     <row r="73" spans="1:29" ht="120" x14ac:dyDescent="0.25">
@@ -8009,7 +8005,7 @@
         <v>674</v>
       </c>
       <c r="U73" s="12" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="V73" s="1" t="s">
         <v>474</v>
@@ -8024,7 +8020,7 @@
         <v>820</v>
       </c>
       <c r="AB73" s="12" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
     </row>
     <row r="74" spans="1:29" ht="405" x14ac:dyDescent="0.25">
@@ -8053,7 +8049,7 @@
         <v>446</v>
       </c>
       <c r="L74" s="2" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="M74" s="2" t="s">
         <v>676</v>
@@ -8083,16 +8079,16 @@
         <v>527</v>
       </c>
       <c r="Y74" s="2" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
       <c r="Z74" s="2" t="s">
         <v>762</v>
       </c>
       <c r="AB74" s="2" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
       <c r="AC74" s="1" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
     </row>
     <row r="75" spans="1:29" ht="45" x14ac:dyDescent="0.25">
@@ -8348,7 +8344,7 @@
         <v>822</v>
       </c>
       <c r="AB79" s="12" t="s">
-        <v>877</v>
+        <v>875</v>
       </c>
     </row>
     <row r="80" spans="1:29" ht="150" x14ac:dyDescent="0.25">
@@ -8737,7 +8733,7 @@
         <v>520</v>
       </c>
       <c r="U86" s="12" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="V86" s="1" t="s">
         <v>474</v>
@@ -8749,13 +8745,13 @@
         <v>527</v>
       </c>
       <c r="Y86" s="2" t="s">
-        <v>826</v>
+        <v>895</v>
       </c>
       <c r="Z86" s="2" t="s">
         <v>710</v>
       </c>
       <c r="AB86" s="12" t="s">
-        <v>843</v>
+        <v>841</v>
       </c>
     </row>
     <row r="87" spans="1:28" ht="150" x14ac:dyDescent="0.25">
@@ -8817,10 +8813,10 @@
         <v>527</v>
       </c>
       <c r="Y87" s="2" t="s">
+        <v>896</v>
+      </c>
+      <c r="AB87" s="12" t="s">
         <v>824</v>
-      </c>
-      <c r="AB87" s="12" t="s">
-        <v>825</v>
       </c>
     </row>
     <row r="88" spans="1:28" ht="150" x14ac:dyDescent="0.25">
@@ -9017,7 +9013,7 @@
         <v>466</v>
       </c>
       <c r="L91" s="14" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
       <c r="M91" s="2" t="s">
         <v>763</v>
@@ -9044,13 +9040,13 @@
         <v>527</v>
       </c>
       <c r="Y91" s="2" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
       <c r="Z91" s="2" t="s">
         <v>765</v>
       </c>
       <c r="AB91" s="12" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
     </row>
     <row r="92" spans="1:28" ht="285" x14ac:dyDescent="0.25">
@@ -9106,13 +9102,13 @@
         <v>527</v>
       </c>
       <c r="Y92" s="2" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="Z92" s="2" t="s">
         <v>765</v>
       </c>
       <c r="AB92" s="12" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
     </row>
     <row r="93" spans="1:28" ht="285" x14ac:dyDescent="0.25">
@@ -9168,13 +9164,13 @@
         <v>527</v>
       </c>
       <c r="Y93" s="2" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="Z93" s="2" t="s">
         <v>765</v>
       </c>
       <c r="AB93" s="12" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
     </row>
     <row r="94" spans="1:28" ht="285" x14ac:dyDescent="0.25">
@@ -9221,7 +9217,7 @@
         <v>727</v>
       </c>
       <c r="U94" s="12" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
       <c r="V94" s="1" t="s">
         <v>474</v>
@@ -9233,7 +9229,7 @@
         <v>527</v>
       </c>
       <c r="Y94" s="2" t="s">
-        <v>832</v>
+        <v>830</v>
       </c>
       <c r="Z94" s="1" t="s">
         <v>766</v>
@@ -9418,13 +9414,13 @@
         <v>527</v>
       </c>
       <c r="Y98" s="2" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
       <c r="Z98" s="2" t="s">
         <v>728</v>
       </c>
       <c r="AB98" s="12" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
     </row>
     <row r="99" spans="1:28" ht="285" x14ac:dyDescent="0.25">
@@ -9471,7 +9467,7 @@
         <v>727</v>
       </c>
       <c r="U99" s="12" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="V99" s="1" t="s">
         <v>474</v>
@@ -9483,13 +9479,13 @@
         <v>527</v>
       </c>
       <c r="Y99" s="2" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="Z99" s="2" t="s">
         <v>734</v>
       </c>
       <c r="AB99" s="12" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
     </row>
     <row r="100" spans="1:28" ht="285" x14ac:dyDescent="0.25">
@@ -9545,13 +9541,13 @@
         <v>527</v>
       </c>
       <c r="Y100" s="2" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
       <c r="Z100" s="2" t="s">
         <v>728</v>
       </c>
       <c r="AB100" s="12" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
     </row>
     <row r="101" spans="1:28" ht="285" x14ac:dyDescent="0.25">
@@ -9607,13 +9603,13 @@
         <v>527</v>
       </c>
       <c r="Y101" s="2" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
       <c r="Z101" s="2" t="s">
         <v>728</v>
       </c>
       <c r="AB101" s="12" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
     </row>
     <row r="102" spans="1:28" ht="150" x14ac:dyDescent="0.25">
@@ -9711,13 +9707,13 @@
         <v>527</v>
       </c>
       <c r="Y103" s="2" t="s">
-        <v>838</v>
+        <v>836</v>
       </c>
       <c r="Z103" s="2" t="s">
         <v>728</v>
       </c>
       <c r="AB103" s="12" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
     </row>
     <row r="104" spans="1:28" ht="150" x14ac:dyDescent="0.25">
@@ -9949,7 +9945,7 @@
         <v>527</v>
       </c>
       <c r="Y108" s="2" t="s">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="Z108" s="2"/>
     </row>
@@ -10006,7 +10002,7 @@
         <v>527</v>
       </c>
       <c r="Y109" s="2" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="Z109" s="2"/>
     </row>
@@ -10281,7 +10277,7 @@
         <v>520</v>
       </c>
       <c r="U114" s="12" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="V114" s="1" t="s">
         <v>474</v>
@@ -10299,7 +10295,7 @@
         <v>753</v>
       </c>
       <c r="AB114" s="12" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
     </row>
     <row r="115" spans="1:28" ht="150" x14ac:dyDescent="0.25">
@@ -10346,7 +10342,7 @@
         <v>520</v>
       </c>
       <c r="U115" s="12" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="V115" s="1" t="s">
         <v>474</v>
@@ -10364,7 +10360,7 @@
         <v>753</v>
       </c>
       <c r="AB115" s="12" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
     </row>
     <row r="116" spans="1:28" ht="45" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
correction CRP and kidney cancer
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-NES.xlsx
+++ b/baseline/data_processing_elements-NES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sbtiali\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maelstrom\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AAEEB5E-2402-491F-9EEE-006B1A0C8ACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49EC0DDE-2EDE-4B67-858B-6C9F0B0A8E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0073E314-1B2C-4924-AC81-D526EEC9786A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{0073E314-1B2C-4924-AC81-D526EEC9786A}"/>
   </bookViews>
   <sheets>
     <sheet name="DPE" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2055" uniqueCount="906">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2056" uniqueCount="908">
   <si>
     <t>index</t>
   </si>
@@ -3352,7 +3352,16 @@
     <t>as.numeric(e31)</t>
   </si>
   <si>
-    <t>as.numeric(e36)</t>
+    <t>The threshold of the machine used for analysis was 4 which is too high to get a proper distribution.</t>
+  </si>
+  <si>
+    <t>cancer_kidney</t>
+  </si>
+  <si>
+    <t>case_when(
+fq113 == 2 ~ 0L;
+cancer_kidney == 1 ~ 1L;
+ELSE ~ NA_integer_ )</t>
   </si>
 </sst>
 </file>
@@ -3828,44 +3837,44 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32FF9666-3C68-4610-B7F3-25EE531D7B07}">
   <dimension ref="A1:AF122"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="5.54296875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.81640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="29" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="40.7109375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="33.5703125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="40.7265625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="33.54296875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="12.1796875" style="1" customWidth="1"/>
     <col min="7" max="7" width="9" style="1"/>
-    <col min="8" max="8" width="14.5703125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="70.7109375" style="2" customWidth="1"/>
-    <col min="10" max="10" width="28.140625" style="2" customWidth="1"/>
-    <col min="11" max="11" width="32.42578125" style="2" customWidth="1"/>
-    <col min="12" max="12" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.54296875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="70.7265625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="28.1796875" style="2" customWidth="1"/>
+    <col min="11" max="11" width="32.453125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="19.54296875" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="42" style="2" customWidth="1"/>
-    <col min="14" max="14" width="14.85546875" style="1" customWidth="1"/>
-    <col min="15" max="15" width="53.7109375" style="2" customWidth="1"/>
-    <col min="16" max="16" width="3.7109375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="4.5703125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="14.81640625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="53.7265625" style="2" customWidth="1"/>
+    <col min="16" max="16" width="3.7265625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="4.54296875" style="1" customWidth="1"/>
     <col min="18" max="18" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="45.85546875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="17.28515625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="32.140625" style="12" customWidth="1"/>
+    <col min="19" max="19" width="45.81640625" style="1" customWidth="1"/>
+    <col min="20" max="20" width="17.26953125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="32.1796875" style="12" customWidth="1"/>
     <col min="22" max="22" width="15" style="1" customWidth="1"/>
-    <col min="23" max="23" width="15.42578125" style="1" customWidth="1"/>
-    <col min="24" max="24" width="16.140625" style="1" customWidth="1"/>
-    <col min="25" max="25" width="49.7109375" style="2" customWidth="1"/>
-    <col min="26" max="26" width="42.28515625" style="1" customWidth="1"/>
-    <col min="27" max="27" width="46.42578125" style="2" customWidth="1"/>
-    <col min="28" max="28" width="54.140625" style="14" customWidth="1"/>
-    <col min="29" max="29" width="39.140625" style="1" customWidth="1"/>
+    <col min="23" max="23" width="15.453125" style="1" customWidth="1"/>
+    <col min="24" max="24" width="16.1796875" style="1" customWidth="1"/>
+    <col min="25" max="25" width="49.7265625" style="2" customWidth="1"/>
+    <col min="26" max="26" width="42.26953125" style="1" customWidth="1"/>
+    <col min="27" max="27" width="46.453125" style="2" customWidth="1"/>
+    <col min="28" max="28" width="54.1796875" style="14" customWidth="1"/>
+    <col min="29" max="29" width="39.1796875" style="1" customWidth="1"/>
     <col min="30" max="30" width="29" style="1" customWidth="1"/>
-    <col min="31" max="31" width="39.140625" style="1" customWidth="1"/>
-    <col min="32" max="32" width="45.28515625" style="1" customWidth="1"/>
+    <col min="31" max="31" width="39.1796875" style="1" customWidth="1"/>
+    <col min="32" max="32" width="45.26953125" style="1" customWidth="1"/>
     <col min="33" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" s="6" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -3963,7 +3972,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -4017,7 +4026,7 @@
       </c>
       <c r="AB2" s="12"/>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -4056,7 +4065,7 @@
       </c>
       <c r="AB3" s="12"/>
     </row>
-    <row r="4" spans="1:32" ht="105" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:32" ht="87" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -4100,7 +4109,7 @@
         <v>774</v>
       </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -4139,7 +4148,7 @@
       </c>
       <c r="AB5" s="12"/>
     </row>
-    <row r="6" spans="1:32" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:32" ht="58" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -4206,7 +4215,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="7" spans="1:32" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:32" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -4259,7 +4268,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="8" spans="1:32" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:32" ht="58" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -4321,7 +4330,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="9" spans="1:32" ht="165" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:32" ht="145" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -4380,7 +4389,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="10" spans="1:32" ht="135" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:32" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -4436,7 +4445,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="11" spans="1:32" ht="75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:32" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -4504,7 +4513,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="12" spans="1:32" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:32" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -4572,7 +4581,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="13" spans="1:32" ht="75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:32" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -4634,7 +4643,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="14" spans="1:32" ht="75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:32" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -4702,7 +4711,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="15" spans="1:32" ht="75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:32" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -4764,7 +4773,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="16" spans="1:32" ht="75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:32" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -4826,7 +4835,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -4888,7 +4897,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -4950,7 +4959,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="90" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" ht="87" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -5018,7 +5027,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -5074,7 +5083,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="90" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" ht="87" x14ac:dyDescent="0.35">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -5139,7 +5148,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -5198,7 +5207,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="180" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:28" ht="174" x14ac:dyDescent="0.35">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -5254,7 +5263,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="105" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" ht="87" x14ac:dyDescent="0.35">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -5316,7 +5325,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="105" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -5369,7 +5378,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:28" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -5410,7 +5419,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="27" spans="1:28" ht="105" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:28" ht="87" x14ac:dyDescent="0.35">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -5472,7 +5481,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="105" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:28" ht="87" x14ac:dyDescent="0.35">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -5531,7 +5540,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="29" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:28" ht="58" x14ac:dyDescent="0.35">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -5593,7 +5602,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="30" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:28" ht="58" x14ac:dyDescent="0.35">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -5652,7 +5661,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="31" spans="1:28" ht="165" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:28" ht="145" x14ac:dyDescent="0.35">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -5714,7 +5723,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="32" spans="1:28" ht="90" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -5776,7 +5785,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="33" spans="1:28" ht="90" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -5838,7 +5847,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="34" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:28" ht="29" x14ac:dyDescent="0.35">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -5876,7 +5885,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="35" spans="1:28" ht="195" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:28" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -5914,7 +5923,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="36" spans="1:28" ht="120" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:28" ht="116" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -5982,7 +5991,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="37" spans="1:28" ht="120" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:28" ht="116" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -6050,7 +6059,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="38" spans="1:28" ht="120" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -6118,7 +6127,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="39" spans="1:28" ht="75" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:28" ht="58" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -6162,7 +6171,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="40" spans="1:28" ht="105" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -6225,7 +6234,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="41" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -6263,7 +6272,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="42" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -6301,7 +6310,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="43" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:28" ht="29" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -6360,7 +6369,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="44" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:28" ht="29" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -6419,7 +6428,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="45" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:28" ht="29" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -6478,7 +6487,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="46" spans="1:28" ht="120" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:28" ht="87" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -6543,7 +6552,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="47" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:28" ht="29" x14ac:dyDescent="0.35">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -6602,7 +6611,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="48" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -6648,20 +6657,23 @@
       <c r="T48" s="1" t="s">
         <v>611</v>
       </c>
+      <c r="U48" s="12" t="s">
+        <v>905</v>
+      </c>
       <c r="V48" s="1" t="s">
-        <v>474</v>
+        <v>513</v>
       </c>
       <c r="W48" s="1" t="s">
-        <v>475</v>
+        <v>512</v>
       </c>
       <c r="X48" s="11" t="s">
-        <v>486</v>
+        <v>513</v>
       </c>
       <c r="Y48" s="11" t="s">
-        <v>905</v>
-      </c>
-    </row>
-    <row r="49" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="49" spans="1:28" ht="29" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -6702,7 +6714,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="50" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -6740,7 +6752,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="51" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:28" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -6781,7 +6793,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="52" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A52" s="1">
         <v>51</v>
       </c>
@@ -6822,7 +6834,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="53" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -6860,7 +6872,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="54" spans="1:28" ht="225" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:28" ht="203" x14ac:dyDescent="0.35">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -6929,7 +6941,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="55" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:28" ht="58" x14ac:dyDescent="0.35">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -6967,7 +6979,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="56" spans="1:28" ht="75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -7032,7 +7044,7 @@
         <v>807</v>
       </c>
     </row>
-    <row r="57" spans="1:28" ht="90" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A57" s="1">
         <v>56</v>
       </c>
@@ -7098,7 +7110,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="58" spans="1:28" ht="90" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A58" s="1">
         <v>57</v>
       </c>
@@ -7166,7 +7178,7 @@
         <v>809</v>
       </c>
     </row>
-    <row r="59" spans="1:28" ht="105" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A59" s="1">
         <v>58</v>
       </c>
@@ -7219,7 +7231,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="60" spans="1:28" ht="165" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:28" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -7278,7 +7290,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="61" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:28" ht="29" x14ac:dyDescent="0.35">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -7316,7 +7328,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="62" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:28" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -7381,7 +7393,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="63" spans="1:28" ht="105" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -7440,7 +7452,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="64" spans="1:28" ht="105" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A64" s="1">
         <v>63</v>
       </c>
@@ -7499,7 +7511,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="65" spans="1:29" ht="180" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:29" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A65" s="1">
         <v>64</v>
       </c>
@@ -7561,7 +7573,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="66" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A66" s="1">
         <v>65</v>
       </c>
@@ -7602,7 +7614,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="67" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:29" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A67" s="1">
         <v>66</v>
       </c>
@@ -7667,7 +7679,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="68" spans="1:29" ht="255" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:29" ht="232" x14ac:dyDescent="0.35">
       <c r="A68" s="1">
         <v>67</v>
       </c>
@@ -7730,7 +7742,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="69" spans="1:29" ht="255" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:29" ht="232" x14ac:dyDescent="0.35">
       <c r="A69" s="1">
         <v>68</v>
       </c>
@@ -7789,7 +7801,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="70" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:29" ht="58" x14ac:dyDescent="0.35">
       <c r="A70" s="1">
         <v>69</v>
       </c>
@@ -7854,7 +7866,7 @@
         <v>813</v>
       </c>
     </row>
-    <row r="71" spans="1:29" ht="105" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:29" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A71" s="1">
         <v>70</v>
       </c>
@@ -7913,7 +7925,7 @@
         <v>866</v>
       </c>
     </row>
-    <row r="72" spans="1:29" ht="90" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:29" ht="87" x14ac:dyDescent="0.35">
       <c r="A72" s="1">
         <v>71</v>
       </c>
@@ -7985,7 +7997,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="73" spans="1:29" ht="120" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:29" ht="87" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
         <v>72</v>
       </c>
@@ -8050,7 +8062,7 @@
         <v>859</v>
       </c>
     </row>
-    <row r="74" spans="1:29" ht="405" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:29" ht="391.5" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
         <v>73</v>
       </c>
@@ -8118,7 +8130,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="75" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:29" ht="29" x14ac:dyDescent="0.35">
       <c r="A75" s="1">
         <v>74</v>
       </c>
@@ -8156,7 +8168,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="76" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A76" s="1">
         <v>75</v>
       </c>
@@ -8194,7 +8206,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="77" spans="1:29" ht="90" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:29" ht="87" x14ac:dyDescent="0.35">
       <c r="A77" s="1">
         <v>76</v>
       </c>
@@ -8247,7 +8259,7 @@
         <v>816</v>
       </c>
     </row>
-    <row r="78" spans="1:29" ht="210" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:29" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A78" s="1">
         <v>77</v>
       </c>
@@ -8309,7 +8321,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="79" spans="1:29" ht="150" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:29" ht="145" x14ac:dyDescent="0.35">
       <c r="A79" s="1">
         <v>78</v>
       </c>
@@ -8374,7 +8386,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="80" spans="1:29" ht="150" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:29" ht="145" x14ac:dyDescent="0.35">
       <c r="A80" s="1">
         <v>79</v>
       </c>
@@ -8433,7 +8445,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="81" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:28" ht="145" x14ac:dyDescent="0.35">
       <c r="A81" s="1">
         <v>80</v>
       </c>
@@ -8477,7 +8489,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="82" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:28" ht="145" x14ac:dyDescent="0.35">
       <c r="A82" s="1">
         <v>81</v>
       </c>
@@ -8536,7 +8548,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="83" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:28" ht="145" x14ac:dyDescent="0.35">
       <c r="A83" s="1">
         <v>82</v>
       </c>
@@ -8595,7 +8607,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="84" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:28" ht="145" x14ac:dyDescent="0.35">
       <c r="A84" s="1">
         <v>83</v>
       </c>
@@ -8654,7 +8666,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="85" spans="1:28" ht="195" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:28" ht="174" x14ac:dyDescent="0.35">
       <c r="A85" s="1">
         <v>84</v>
       </c>
@@ -8713,7 +8725,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="86" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A86" s="1">
         <v>85</v>
       </c>
@@ -8781,7 +8793,7 @@
         <v>836</v>
       </c>
     </row>
-    <row r="87" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:28" ht="145" x14ac:dyDescent="0.35">
       <c r="A87" s="1">
         <v>86</v>
       </c>
@@ -8846,7 +8858,7 @@
         <v>819</v>
       </c>
     </row>
-    <row r="88" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:28" ht="145" x14ac:dyDescent="0.35">
       <c r="A88" s="1">
         <v>87</v>
       </c>
@@ -8905,7 +8917,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="89" spans="1:28" ht="60" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:28" ht="58" x14ac:dyDescent="0.35">
       <c r="A89" s="1">
         <v>88</v>
       </c>
@@ -8958,7 +8970,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="90" spans="1:28" ht="105" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
       <c r="A90" s="1">
         <v>89</v>
       </c>
@@ -9014,7 +9026,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="91" spans="1:28" ht="285" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A91" s="1">
         <v>90</v>
       </c>
@@ -9076,7 +9088,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="92" spans="1:28" ht="285" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A92" s="1">
         <v>91</v>
       </c>
@@ -9138,7 +9150,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="93" spans="1:28" ht="285" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A93" s="1">
         <v>92</v>
       </c>
@@ -9200,7 +9212,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="94" spans="1:28" ht="285" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A94" s="1">
         <v>93</v>
       </c>
@@ -9262,7 +9274,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="95" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A95" s="1">
         <v>94</v>
       </c>
@@ -9288,23 +9300,23 @@
         <v>466</v>
       </c>
       <c r="L95" s="1" t="s">
-        <v>477</v>
+        <v>906</v>
       </c>
       <c r="V95" s="1" t="s">
-        <v>513</v>
+        <v>474</v>
       </c>
       <c r="W95" s="1" t="s">
-        <v>546</v>
+        <v>500</v>
       </c>
       <c r="X95" s="1" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
       <c r="Y95" s="2" t="s">
-        <v>513</v>
+        <v>907</v>
       </c>
       <c r="Z95" s="2"/>
     </row>
-    <row r="96" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A96" s="1">
         <v>95</v>
       </c>
@@ -9346,7 +9358,7 @@
       </c>
       <c r="Z96" s="2"/>
     </row>
-    <row r="97" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A97" s="1">
         <v>96</v>
       </c>
@@ -9388,7 +9400,7 @@
       </c>
       <c r="Z97" s="2"/>
     </row>
-    <row r="98" spans="1:28" ht="285" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A98" s="1">
         <v>97</v>
       </c>
@@ -9450,7 +9462,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="99" spans="1:28" ht="285" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A99" s="1">
         <v>98</v>
       </c>
@@ -9515,7 +9527,7 @@
         <v>856</v>
       </c>
     </row>
-    <row r="100" spans="1:28" ht="285" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A100" s="1">
         <v>99</v>
       </c>
@@ -9577,7 +9589,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="101" spans="1:28" ht="285" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A101" s="1">
         <v>100</v>
       </c>
@@ -9639,7 +9651,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="102" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A102" s="1">
         <v>101</v>
       </c>
@@ -9681,7 +9693,7 @@
       </c>
       <c r="Z102" s="2"/>
     </row>
-    <row r="103" spans="1:28" ht="285" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A103" s="1">
         <v>102</v>
       </c>
@@ -9743,7 +9755,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="104" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A104" s="1">
         <v>103</v>
       </c>
@@ -9787,7 +9799,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="105" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A105" s="1">
         <v>104</v>
       </c>
@@ -9831,7 +9843,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="106" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A106" s="1">
         <v>105</v>
       </c>
@@ -9875,7 +9887,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="107" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A107" s="1">
         <v>106</v>
       </c>
@@ -9919,7 +9931,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="108" spans="1:28" ht="285" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A108" s="1">
         <v>107</v>
       </c>
@@ -9976,7 +9988,7 @@
       </c>
       <c r="Z108" s="2"/>
     </row>
-    <row r="109" spans="1:28" ht="285" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
       <c r="A109" s="1">
         <v>108</v>
       </c>
@@ -10033,7 +10045,7 @@
       </c>
       <c r="Z109" s="2"/>
     </row>
-    <row r="110" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:28" ht="145" x14ac:dyDescent="0.35">
       <c r="A110" s="1">
         <v>109</v>
       </c>
@@ -10089,7 +10101,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="111" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:28" ht="145" x14ac:dyDescent="0.35">
       <c r="A111" s="1">
         <v>110</v>
       </c>
@@ -10145,7 +10157,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="112" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:28" ht="145" x14ac:dyDescent="0.35">
       <c r="A112" s="1">
         <v>111</v>
       </c>
@@ -10201,7 +10213,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="113" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:28" ht="145" x14ac:dyDescent="0.35">
       <c r="A113" s="1">
         <v>112</v>
       </c>
@@ -10260,7 +10272,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="114" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:28" ht="145" x14ac:dyDescent="0.35">
       <c r="A114" s="1">
         <v>113</v>
       </c>
@@ -10325,7 +10337,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="115" spans="1:28" ht="150" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:28" ht="145" x14ac:dyDescent="0.35">
       <c r="A115" s="1">
         <v>114</v>
       </c>
@@ -10390,7 +10402,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="116" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A116" s="1">
         <v>115</v>
       </c>
@@ -10428,7 +10440,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="117" spans="1:28" ht="45" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A117" s="1">
         <v>116</v>
       </c>
@@ -10466,7 +10478,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="118" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A118" s="1">
         <v>117</v>
       </c>
@@ -10504,7 +10516,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="119" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:28" ht="29" x14ac:dyDescent="0.35">
       <c r="A119" s="1">
         <v>118</v>
       </c>
@@ -10542,7 +10554,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="120" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:28" ht="29" x14ac:dyDescent="0.35">
       <c r="A120" s="1">
         <v>119</v>
       </c>
@@ -10580,7 +10592,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="121" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:28" ht="29" x14ac:dyDescent="0.35">
       <c r="A121" s="1">
         <v>120</v>
       </c>
@@ -10618,7 +10630,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="122" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:28" ht="29" x14ac:dyDescent="0.35">
       <c r="A122" s="1">
         <v>121</v>
       </c>

</xml_diff>

<commit_message>
add cancer type variables
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-NES.xlsx
+++ b/baseline/data_processing_elements-NES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maelstrom\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49EC0DDE-2EDE-4B67-858B-6C9F0B0A8E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFA726EF-D272-4874-9852-F0D7C7A0344C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{0073E314-1B2C-4924-AC81-D526EEC9786A}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2056" uniqueCount="908">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2056" uniqueCount="914">
   <si>
     <t>index</t>
   </si>
@@ -3355,12 +3355,39 @@
     <t>The threshold of the machine used for analysis was 4 which is too high to get a proper distribution.</t>
   </si>
   <si>
-    <t>cancer_kidney</t>
+    <t>cancer_type_throat</t>
   </si>
   <si>
     <t>case_when(
 fq113 == 2 ~ 0L;
-cancer_kidney == 1 ~ 1L;
+cancer_type_throat == 1 ~ 1L;
+ELSE ~ NA_integer_ )</t>
+  </si>
+  <si>
+    <t>case_when(
+fq113 == 2 ~ 0L;
+cancer_type_kidney == 1 ~ 1L;
+ELSE ~ NA_integer_ )</t>
+  </si>
+  <si>
+    <t>cancer_type_kidney</t>
+  </si>
+  <si>
+    <t>cancer_type_leukaemia</t>
+  </si>
+  <si>
+    <t>case_when(
+fq113 == 2 ~ 0L;
+cancer_type_leukaemia == 1 ~ 1L;
+ELSE ~ NA_integer_ )</t>
+  </si>
+  <si>
+    <t>cancer_type_uterus</t>
+  </si>
+  <si>
+    <t>case_when(
+fq113 == 2 ~ 0L;
+cancer_type_uterus == 1 ~ 1L;
 ELSE ~ NA_integer_ )</t>
   </si>
 </sst>
@@ -9300,7 +9327,7 @@
         <v>466</v>
       </c>
       <c r="L95" s="1" t="s">
-        <v>906</v>
+        <v>909</v>
       </c>
       <c r="V95" s="1" t="s">
         <v>474</v>
@@ -9312,7 +9339,7 @@
         <v>526</v>
       </c>
       <c r="Y95" s="2" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="Z95" s="2"/>
     </row>
@@ -9342,19 +9369,19 @@
         <v>466</v>
       </c>
       <c r="L96" s="1" t="s">
-        <v>477</v>
+        <v>906</v>
       </c>
       <c r="V96" s="1" t="s">
-        <v>513</v>
+        <v>474</v>
       </c>
       <c r="W96" s="1" t="s">
-        <v>546</v>
+        <v>500</v>
       </c>
       <c r="X96" s="1" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
       <c r="Y96" s="2" t="s">
-        <v>513</v>
+        <v>907</v>
       </c>
       <c r="Z96" s="2"/>
     </row>
@@ -9384,19 +9411,19 @@
         <v>466</v>
       </c>
       <c r="L97" s="1" t="s">
-        <v>477</v>
+        <v>910</v>
       </c>
       <c r="V97" s="1" t="s">
-        <v>513</v>
+        <v>474</v>
       </c>
       <c r="W97" s="1" t="s">
-        <v>546</v>
+        <v>500</v>
       </c>
       <c r="X97" s="1" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
       <c r="Y97" s="2" t="s">
-        <v>513</v>
+        <v>911</v>
       </c>
       <c r="Z97" s="2"/>
     </row>
@@ -9746,7 +9773,7 @@
         <v>526</v>
       </c>
       <c r="Y103" s="2" t="s">
-        <v>831</v>
+        <v>913</v>
       </c>
       <c r="Z103" s="2" t="s">
         <v>727</v>
@@ -9781,19 +9808,19 @@
         <v>466</v>
       </c>
       <c r="L104" s="1" t="s">
-        <v>477</v>
+        <v>912</v>
       </c>
       <c r="V104" s="1" t="s">
-        <v>513</v>
+        <v>474</v>
       </c>
       <c r="W104" s="1" t="s">
-        <v>546</v>
+        <v>500</v>
       </c>
       <c r="X104" s="1" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
       <c r="Y104" s="2" t="s">
-        <v>513</v>
+        <v>831</v>
       </c>
       <c r="Z104" s="2" t="s">
         <v>736</v>

</xml_diff>

<commit_message>
correct msk and age
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-NES.xlsx
+++ b/baseline/data_processing_elements-NES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maelstrom\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFA726EF-D272-4874-9852-F0D7C7A0344C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F94A739F-3AA6-4FC5-AB27-E5EFEB875E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{0073E314-1B2C-4924-AC81-D526EEC9786A}"/>
   </bookViews>
@@ -3291,17 +3291,8 @@
 ELSE ~ NA_integer_)</t>
   </si>
   <si>
-    <t>case_when(
-fq289 == 1 | fq319 == 1 | fq364 == 1 ~ 1L;
-fq289 == 2 &amp; fq319 == 2 &amp; fq364 ==0 ~ 0L ; 
-ELSE ~ NA_integer_)</t>
-  </si>
-  <si>
     <t>questionnaire_date;
 bq2</t>
-  </si>
-  <si>
-    <t>lubridate::interval(as.Date(questionnaire_date), as.Date(bq2)) %/% lubridate::years(1)</t>
   </si>
   <si>
     <t>as.numeric(e32)</t>
@@ -3389,6 +3380,15 @@
 fq113 == 2 ~ 0L;
 cancer_type_uterus == 1 ~ 1L;
 ELSE ~ NA_integer_ )</t>
+  </si>
+  <si>
+    <t>case_when(
+fq289 == 1 | fq319 == 1 | fq364 == 1 ~ 1L;
+fq289 == 2 &amp; fq319 == 2 &amp; fq364 ==2 ~ 0L ; 
+ELSE ~ NA_integer_)</t>
+  </si>
+  <si>
+    <t>lubridate::interval(as.Date(bq2),as.Date(questionnaire_date)) %/% lubridate::years(1)</t>
   </si>
 </sst>
 </file>
@@ -4321,7 +4321,7 @@
         <v>396</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="M8" s="2" t="s">
         <v>494</v>
@@ -4351,7 +4351,7 @@
         <v>486</v>
       </c>
       <c r="Y8" s="2" t="s">
-        <v>890</v>
+        <v>913</v>
       </c>
       <c r="AB8" s="12" t="s">
         <v>778</v>
@@ -5228,7 +5228,7 @@
         <v>486</v>
       </c>
       <c r="Y22" s="2" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
       <c r="AB22" s="12" t="s">
         <v>870</v>
@@ -5502,7 +5502,7 @@
         <v>486</v>
       </c>
       <c r="Y27" s="12" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="AB27" s="12" t="s">
         <v>792</v>
@@ -5623,7 +5623,7 @@
         <v>486</v>
       </c>
       <c r="Y29" s="11" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
       <c r="AB29" s="12" t="s">
         <v>795</v>
@@ -5682,7 +5682,7 @@
         <v>526</v>
       </c>
       <c r="Y30" s="12" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
       <c r="AB30" s="12" t="s">
         <v>794</v>
@@ -5744,7 +5744,7 @@
         <v>486</v>
       </c>
       <c r="Y31" s="12" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="AB31" s="12" t="s">
         <v>796</v>
@@ -5806,7 +5806,7 @@
         <v>486</v>
       </c>
       <c r="Y32" s="12" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
       <c r="AB32" s="12" t="s">
         <v>795</v>
@@ -5865,7 +5865,7 @@
         <v>526</v>
       </c>
       <c r="Y33" s="12" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="Z33" s="2" t="s">
         <v>564</v>
@@ -5909,7 +5909,7 @@
         <v>486</v>
       </c>
       <c r="Y34" s="1" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
     </row>
     <row r="35" spans="1:28" ht="159.5" x14ac:dyDescent="0.35">
@@ -5944,7 +5944,7 @@
         <v>526</v>
       </c>
       <c r="Y35" s="2" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="Z35" s="2" t="s">
         <v>885</v>
@@ -6145,7 +6145,7 @@
         <v>486</v>
       </c>
       <c r="Y38" s="12" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="Z38" s="2" t="s">
         <v>569</v>
@@ -6390,7 +6390,7 @@
         <v>486</v>
       </c>
       <c r="Y43" s="1" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
       <c r="AB43" s="12" t="s">
         <v>850</v>
@@ -6449,7 +6449,7 @@
         <v>486</v>
       </c>
       <c r="Y44" s="1" t="s">
-        <v>903</v>
+        <v>901</v>
       </c>
       <c r="AB44" s="12" t="s">
         <v>850</v>
@@ -6508,7 +6508,7 @@
         <v>486</v>
       </c>
       <c r="Y45" s="1" t="s">
-        <v>904</v>
+        <v>902</v>
       </c>
       <c r="AB45" s="12" t="s">
         <v>850</v>
@@ -6632,7 +6632,7 @@
         <v>486</v>
       </c>
       <c r="Y47" s="11" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="AB47" s="12" t="s">
         <v>850</v>
@@ -6685,7 +6685,7 @@
         <v>611</v>
       </c>
       <c r="U48" s="12" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="V48" s="1" t="s">
         <v>513</v>
@@ -8879,7 +8879,7 @@
         <v>526</v>
       </c>
       <c r="Y87" s="2" t="s">
-        <v>888</v>
+        <v>912</v>
       </c>
       <c r="AB87" s="12" t="s">
         <v>819</v>
@@ -9327,7 +9327,7 @@
         <v>466</v>
       </c>
       <c r="L95" s="1" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
       <c r="V95" s="1" t="s">
         <v>474</v>
@@ -9339,7 +9339,7 @@
         <v>526</v>
       </c>
       <c r="Y95" s="2" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="Z95" s="2"/>
     </row>
@@ -9369,7 +9369,7 @@
         <v>466</v>
       </c>
       <c r="L96" s="1" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="V96" s="1" t="s">
         <v>474</v>
@@ -9381,7 +9381,7 @@
         <v>526</v>
       </c>
       <c r="Y96" s="2" t="s">
-        <v>907</v>
+        <v>905</v>
       </c>
       <c r="Z96" s="2"/>
     </row>
@@ -9411,7 +9411,7 @@
         <v>466</v>
       </c>
       <c r="L97" s="1" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="V97" s="1" t="s">
         <v>474</v>
@@ -9423,7 +9423,7 @@
         <v>526</v>
       </c>
       <c r="Y97" s="2" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
       <c r="Z97" s="2"/>
     </row>
@@ -9773,7 +9773,7 @@
         <v>526</v>
       </c>
       <c r="Y103" s="2" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
       <c r="Z103" s="2" t="s">
         <v>727</v>
@@ -9808,7 +9808,7 @@
         <v>466</v>
       </c>
       <c r="L104" s="1" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="V104" s="1" t="s">
         <v>474</v>

</xml_diff>

<commit_message>
correcting resting heart rate
</commit_message>
<xml_diff>
--- a/baseline/data_processing_elements-NES.xlsx
+++ b/baseline/data_processing_elements-NES.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maelstrom\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F94A739F-3AA6-4FC5-AB27-E5EFEB875E93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A0385C-A6E2-485F-A499-C9768AB9458D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{0073E314-1B2C-4924-AC81-D526EEC9786A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{0073E314-1B2C-4924-AC81-D526EEC9786A}"/>
   </bookViews>
   <sheets>
     <sheet name="DPE" sheetId="1" r:id="rId1"/>
@@ -3331,9 +3331,6 @@
 ELSE ~ NA)</t>
   </si>
   <si>
-    <t>(as.numeric(e9) + as.numeric(e13) + as.numeric(e17) + as.numeric(e21)) %&gt;% round(., 0)</t>
-  </si>
-  <si>
     <t>as.numeric(e29)</t>
   </si>
   <si>
@@ -3389,6 +3386,15 @@
   </si>
   <si>
     <t>lubridate::interval(as.Date(bq2),as.Date(questionnaire_date)) %/% lubridate::years(1)</t>
+  </si>
+  <si>
+    <t>round(rowMeans(
+mutate(.,
+e9_temp = as.numeric(e9),
+e13_temp = as.numeric(e13),
+e17_temp = as.numeric(e17),
+e21_temp = as.numeric(e21)) %&gt;% 
+select(e9_temp, e13_temp, e17_temp, e21_temp), na.rm = TRUE), 0)</t>
   </si>
 </sst>
 </file>
@@ -3547,7 +3553,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -3864,44 +3870,44 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32FF9666-3C68-4610-B7F3-25EE531D7B07}">
   <dimension ref="A1:AF122"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.54296875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.81640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="5.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="29" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="40.7265625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="33.54296875" style="2" customWidth="1"/>
-    <col min="6" max="6" width="12.1796875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="40.7109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="33.5703125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" style="1" customWidth="1"/>
     <col min="7" max="7" width="9" style="1"/>
-    <col min="8" max="8" width="14.54296875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="70.7265625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="28.1796875" style="2" customWidth="1"/>
-    <col min="11" max="11" width="32.453125" style="2" customWidth="1"/>
-    <col min="12" max="12" width="19.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="70.7109375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="28.140625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="32.42578125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="42" style="2" customWidth="1"/>
-    <col min="14" max="14" width="14.81640625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="53.7265625" style="2" customWidth="1"/>
-    <col min="16" max="16" width="3.7265625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="4.54296875" style="1" customWidth="1"/>
+    <col min="14" max="14" width="14.85546875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="53.7109375" style="2" customWidth="1"/>
+    <col min="16" max="16" width="3.7109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="4.5703125" style="1" customWidth="1"/>
     <col min="18" max="18" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="45.81640625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="17.26953125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="32.1796875" style="12" customWidth="1"/>
+    <col min="19" max="19" width="45.85546875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="17.28515625" style="1" customWidth="1"/>
+    <col min="21" max="21" width="32.140625" style="12" customWidth="1"/>
     <col min="22" max="22" width="15" style="1" customWidth="1"/>
-    <col min="23" max="23" width="15.453125" style="1" customWidth="1"/>
-    <col min="24" max="24" width="16.1796875" style="1" customWidth="1"/>
-    <col min="25" max="25" width="49.7265625" style="2" customWidth="1"/>
-    <col min="26" max="26" width="42.26953125" style="1" customWidth="1"/>
-    <col min="27" max="27" width="46.453125" style="2" customWidth="1"/>
-    <col min="28" max="28" width="54.1796875" style="14" customWidth="1"/>
-    <col min="29" max="29" width="39.1796875" style="1" customWidth="1"/>
+    <col min="23" max="23" width="15.42578125" style="1" customWidth="1"/>
+    <col min="24" max="24" width="16.140625" style="1" customWidth="1"/>
+    <col min="25" max="25" width="49.7109375" style="2" customWidth="1"/>
+    <col min="26" max="26" width="42.28515625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="46.42578125" style="2" customWidth="1"/>
+    <col min="28" max="28" width="54.140625" style="14" customWidth="1"/>
+    <col min="29" max="29" width="39.140625" style="1" customWidth="1"/>
     <col min="30" max="30" width="29" style="1" customWidth="1"/>
-    <col min="31" max="31" width="39.1796875" style="1" customWidth="1"/>
-    <col min="32" max="32" width="45.26953125" style="1" customWidth="1"/>
+    <col min="31" max="31" width="39.140625" style="1" customWidth="1"/>
+    <col min="32" max="32" width="45.28515625" style="1" customWidth="1"/>
     <col min="33" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" s="6" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:32" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -3999,7 +4005,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -4053,7 +4059,7 @@
       </c>
       <c r="AB2" s="12"/>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -4092,7 +4098,7 @@
       </c>
       <c r="AB3" s="12"/>
     </row>
-    <row r="4" spans="1:32" ht="87" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:32" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -4136,7 +4142,7 @@
         <v>774</v>
       </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -4175,7 +4181,7 @@
       </c>
       <c r="AB5" s="12"/>
     </row>
-    <row r="6" spans="1:32" ht="58" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:32" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -4242,7 +4248,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="7" spans="1:32" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:32" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -4295,7 +4301,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="8" spans="1:32" ht="58" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:32" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -4351,13 +4357,13 @@
         <v>486</v>
       </c>
       <c r="Y8" s="2" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="AB8" s="12" t="s">
         <v>778</v>
       </c>
     </row>
-    <row r="9" spans="1:32" ht="145" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:32" ht="165" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -4416,7 +4422,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="10" spans="1:32" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:32" ht="135" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -4472,7 +4478,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="11" spans="1:32" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:32" ht="75" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -4540,7 +4546,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="12" spans="1:32" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:32" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -4608,7 +4614,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="13" spans="1:32" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:32" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -4670,7 +4676,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="14" spans="1:32" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:32" ht="75" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -4738,7 +4744,7 @@
         <v>788</v>
       </c>
     </row>
-    <row r="15" spans="1:32" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:32" ht="75" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -4800,7 +4806,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="16" spans="1:32" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:32" ht="75" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -4862,7 +4868,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="17" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -4924,7 +4930,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="18" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -4986,7 +4992,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="19" spans="1:28" ht="87" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -5054,7 +5060,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="20" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -5110,7 +5116,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="21" spans="1:28" ht="87" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -5175,7 +5181,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="22" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -5234,7 +5240,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="23" spans="1:28" ht="174" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:28" ht="180" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -5290,7 +5296,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="24" spans="1:28" ht="87" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:28" ht="105" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -5352,7 +5358,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="25" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:28" ht="105" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -5405,7 +5411,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="26" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -5446,7 +5452,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="27" spans="1:28" ht="87" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:28" ht="105" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -5508,7 +5514,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="28" spans="1:28" ht="87" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:28" ht="105" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -5567,7 +5573,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="29" spans="1:28" ht="58" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -5629,7 +5635,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="30" spans="1:28" ht="58" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -5688,7 +5694,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="31" spans="1:28" ht="145" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:28" ht="165" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -5750,7 +5756,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="32" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -5812,7 +5818,7 @@
         <v>795</v>
       </c>
     </row>
-    <row r="33" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -5874,7 +5880,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="34" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -5912,7 +5918,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="35" spans="1:28" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:28" ht="195" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -5950,7 +5956,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="36" spans="1:28" ht="116" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:28" ht="120" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -6018,7 +6024,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="37" spans="1:28" ht="116" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:28" ht="120" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -6086,7 +6092,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="38" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:28" ht="120" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -6145,7 +6151,7 @@
         <v>486</v>
       </c>
       <c r="Y38" s="12" t="s">
-        <v>899</v>
+        <v>913</v>
       </c>
       <c r="Z38" s="2" t="s">
         <v>569</v>
@@ -6154,7 +6160,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="39" spans="1:28" ht="58" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -6198,7 +6204,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="40" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:28" ht="105" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -6261,7 +6267,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="41" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -6299,7 +6305,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="42" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>41</v>
       </c>
@@ -6337,7 +6343,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="43" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>42</v>
       </c>
@@ -6390,13 +6396,13 @@
         <v>486</v>
       </c>
       <c r="Y43" s="1" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="AB43" s="12" t="s">
         <v>850</v>
       </c>
     </row>
-    <row r="44" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>43</v>
       </c>
@@ -6449,13 +6455,13 @@
         <v>486</v>
       </c>
       <c r="Y44" s="1" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="AB44" s="12" t="s">
         <v>850</v>
       </c>
     </row>
-    <row r="45" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>44</v>
       </c>
@@ -6508,13 +6514,13 @@
         <v>486</v>
       </c>
       <c r="Y45" s="1" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="AB45" s="12" t="s">
         <v>850</v>
       </c>
     </row>
-    <row r="46" spans="1:28" ht="87" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:28" ht="120" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>45</v>
       </c>
@@ -6579,7 +6585,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="47" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>46</v>
       </c>
@@ -6638,7 +6644,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="48" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>47</v>
       </c>
@@ -6685,7 +6691,7 @@
         <v>611</v>
       </c>
       <c r="U48" s="12" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="V48" s="1" t="s">
         <v>513</v>
@@ -6700,7 +6706,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="49" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>48</v>
       </c>
@@ -6741,7 +6747,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="50" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>49</v>
       </c>
@@ -6779,7 +6785,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="51" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>50</v>
       </c>
@@ -6820,7 +6826,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="52" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>51</v>
       </c>
@@ -6861,7 +6867,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="53" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>52</v>
       </c>
@@ -6899,7 +6905,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="54" spans="1:28" ht="203" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:28" ht="225" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>53</v>
       </c>
@@ -6968,7 +6974,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="55" spans="1:28" ht="58" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>54</v>
       </c>
@@ -7006,7 +7012,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="56" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:28" ht="75" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>55</v>
       </c>
@@ -7071,7 +7077,7 @@
         <v>807</v>
       </c>
     </row>
-    <row r="57" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>56</v>
       </c>
@@ -7137,7 +7143,7 @@
         <v>853</v>
       </c>
     </row>
-    <row r="58" spans="1:28" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:28" ht="90" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>57</v>
       </c>
@@ -7205,7 +7211,7 @@
         <v>809</v>
       </c>
     </row>
-    <row r="59" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:28" ht="105" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>58</v>
       </c>
@@ -7258,7 +7264,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="60" spans="1:28" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:28" ht="165" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>59</v>
       </c>
@@ -7317,7 +7323,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="61" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
         <v>60</v>
       </c>
@@ -7355,7 +7361,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="62" spans="1:28" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:28" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>61</v>
       </c>
@@ -7420,7 +7426,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="63" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:28" ht="105" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>62</v>
       </c>
@@ -7479,7 +7485,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="64" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:28" ht="105" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>63</v>
       </c>
@@ -7538,7 +7544,7 @@
         <v>810</v>
       </c>
     </row>
-    <row r="65" spans="1:29" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:29" ht="180" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>64</v>
       </c>
@@ -7600,7 +7606,7 @@
         <v>862</v>
       </c>
     </row>
-    <row r="66" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>65</v>
       </c>
@@ -7641,7 +7647,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="67" spans="1:29" ht="409.5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:29" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
         <v>66</v>
       </c>
@@ -7706,7 +7712,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="68" spans="1:29" ht="232" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:29" ht="255" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>67</v>
       </c>
@@ -7769,7 +7775,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="69" spans="1:29" ht="232" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:29" ht="255" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>68</v>
       </c>
@@ -7828,7 +7834,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="70" spans="1:29" ht="58" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>69</v>
       </c>
@@ -7893,7 +7899,7 @@
         <v>813</v>
       </c>
     </row>
-    <row r="71" spans="1:29" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:29" ht="105" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>70</v>
       </c>
@@ -7952,7 +7958,7 @@
         <v>866</v>
       </c>
     </row>
-    <row r="72" spans="1:29" ht="87" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:29" ht="90" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>71</v>
       </c>
@@ -8024,7 +8030,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="73" spans="1:29" ht="87" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:29" ht="120" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>72</v>
       </c>
@@ -8089,7 +8095,7 @@
         <v>859</v>
       </c>
     </row>
-    <row r="74" spans="1:29" ht="391.5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:29" ht="405" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>73</v>
       </c>
@@ -8157,7 +8163,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="75" spans="1:29" ht="29" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
         <v>74</v>
       </c>
@@ -8195,7 +8201,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="76" spans="1:29" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>75</v>
       </c>
@@ -8233,7 +8239,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="77" spans="1:29" ht="87" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:29" ht="90" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>76</v>
       </c>
@@ -8286,7 +8292,7 @@
         <v>816</v>
       </c>
     </row>
-    <row r="78" spans="1:29" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:29" ht="210" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
         <v>77</v>
       </c>
@@ -8348,7 +8354,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="79" spans="1:29" ht="145" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:29" ht="150" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>78</v>
       </c>
@@ -8413,7 +8419,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="80" spans="1:29" ht="145" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:29" ht="150" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>79</v>
       </c>
@@ -8472,7 +8478,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="81" spans="1:28" ht="145" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>80</v>
       </c>
@@ -8516,7 +8522,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="82" spans="1:28" ht="145" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>81</v>
       </c>
@@ -8575,7 +8581,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="83" spans="1:28" ht="145" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>82</v>
       </c>
@@ -8634,7 +8640,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="84" spans="1:28" ht="145" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
         <v>83</v>
       </c>
@@ -8693,7 +8699,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="85" spans="1:28" ht="174" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:28" ht="180" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
         <v>84</v>
       </c>
@@ -8752,7 +8758,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="86" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
         <v>85</v>
       </c>
@@ -8820,7 +8826,7 @@
         <v>836</v>
       </c>
     </row>
-    <row r="87" spans="1:28" ht="145" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>86</v>
       </c>
@@ -8879,13 +8885,13 @@
         <v>526</v>
       </c>
       <c r="Y87" s="2" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="AB87" s="12" t="s">
         <v>819</v>
       </c>
     </row>
-    <row r="88" spans="1:28" ht="145" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>87</v>
       </c>
@@ -8944,7 +8950,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="89" spans="1:28" ht="58" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:28" ht="60" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
         <v>88</v>
       </c>
@@ -8997,7 +9003,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="90" spans="1:28" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:28" ht="105" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
         <v>89</v>
       </c>
@@ -9053,7 +9059,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="91" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:28" ht="285" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>90</v>
       </c>
@@ -9115,7 +9121,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="92" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:28" ht="285" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
         <v>91</v>
       </c>
@@ -9177,7 +9183,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="93" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:28" ht="285" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
         <v>92</v>
       </c>
@@ -9239,7 +9245,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="94" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:28" ht="285" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>93</v>
       </c>
@@ -9301,7 +9307,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="95" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
         <v>94</v>
       </c>
@@ -9327,7 +9333,7 @@
         <v>466</v>
       </c>
       <c r="L95" s="1" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="V95" s="1" t="s">
         <v>474</v>
@@ -9339,11 +9345,11 @@
         <v>526</v>
       </c>
       <c r="Y95" s="2" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="Z95" s="2"/>
     </row>
-    <row r="96" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>95</v>
       </c>
@@ -9369,7 +9375,7 @@
         <v>466</v>
       </c>
       <c r="L96" s="1" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="V96" s="1" t="s">
         <v>474</v>
@@ -9381,11 +9387,11 @@
         <v>526</v>
       </c>
       <c r="Y96" s="2" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="Z96" s="2"/>
     </row>
-    <row r="97" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>96</v>
       </c>
@@ -9411,7 +9417,7 @@
         <v>466</v>
       </c>
       <c r="L97" s="1" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="V97" s="1" t="s">
         <v>474</v>
@@ -9423,11 +9429,11 @@
         <v>526</v>
       </c>
       <c r="Y97" s="2" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="Z97" s="2"/>
     </row>
-    <row r="98" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:28" ht="285" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>97</v>
       </c>
@@ -9489,7 +9495,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="99" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:28" ht="285" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>98</v>
       </c>
@@ -9554,7 +9560,7 @@
         <v>856</v>
       </c>
     </row>
-    <row r="100" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:28" ht="285" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>99</v>
       </c>
@@ -9616,7 +9622,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="101" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:28" ht="285" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>100</v>
       </c>
@@ -9678,7 +9684,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="102" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>101</v>
       </c>
@@ -9720,7 +9726,7 @@
       </c>
       <c r="Z102" s="2"/>
     </row>
-    <row r="103" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:28" ht="285" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
         <v>102</v>
       </c>
@@ -9773,7 +9779,7 @@
         <v>526</v>
       </c>
       <c r="Y103" s="2" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="Z103" s="2" t="s">
         <v>727</v>
@@ -9782,7 +9788,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="104" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>103</v>
       </c>
@@ -9808,7 +9814,7 @@
         <v>466</v>
       </c>
       <c r="L104" s="1" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="V104" s="1" t="s">
         <v>474</v>
@@ -9826,7 +9832,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="105" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
         <v>104</v>
       </c>
@@ -9870,7 +9876,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="106" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
         <v>105</v>
       </c>
@@ -9914,7 +9920,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="107" spans="1:28" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
         <v>106</v>
       </c>
@@ -9958,7 +9964,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="108" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:28" ht="285" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
         <v>107</v>
       </c>
@@ -10015,7 +10021,7 @@
       </c>
       <c r="Z108" s="2"/>
     </row>
-    <row r="109" spans="1:28" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:28" ht="285" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
         <v>108</v>
       </c>
@@ -10072,7 +10078,7 @@
       </c>
       <c r="Z109" s="2"/>
     </row>
-    <row r="110" spans="1:28" ht="145" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
         <v>109</v>
       </c>
@@ -10128,7 +10134,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="111" spans="1:28" ht="145" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
         <v>110</v>
       </c>
@@ -10184,7 +10190,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="112" spans="1:28" ht="145" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
         <v>111</v>
       </c>
@@ -10240,7 +10246,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="113" spans="1:28" ht="145" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A113" s="1">
         <v>112</v>
       </c>
@@ -10299,7 +10305,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="114" spans="1:28" ht="145" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A114" s="1">
         <v>113</v>
       </c>
@@ -10364,7 +10370,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="115" spans="1:28" ht="145" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:28" ht="150" x14ac:dyDescent="0.25">
       <c r="A115" s="1">
         <v>114</v>
       </c>
@@ -10429,7 +10435,7 @@
         <v>834</v>
       </c>
     </row>
-    <row r="116" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A116" s="1">
         <v>115</v>
       </c>
@@ -10467,7 +10473,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="117" spans="1:28" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:28" ht="45" x14ac:dyDescent="0.25">
       <c r="A117" s="1">
         <v>116</v>
       </c>
@@ -10505,7 +10511,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="118" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A118" s="1">
         <v>117</v>
       </c>
@@ -10543,7 +10549,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="119" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A119" s="1">
         <v>118</v>
       </c>
@@ -10581,7 +10587,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="120" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A120" s="1">
         <v>119</v>
       </c>
@@ -10619,7 +10625,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="121" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A121" s="1">
         <v>120</v>
       </c>
@@ -10657,7 +10663,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="122" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A122" s="1">
         <v>121</v>
       </c>

</xml_diff>